<commit_message>
Set data cut-off to 14-Aug-2026 and update conclusions
- Prices, betas, 52-week ranges and NTPC Green value as of the 14-Aug-2026 close
- G-sec 6.76% (14-Aug close); stub period 229/365
- Consensus rebuilt from broker targets dated on or before 14-Aug-2026
- NTPC HOLD 314, Tata Power SELL 331, JSW Energy HOLD 506 (borderline)
</commit_message>
<xml_diff>
--- a/outputs/JSWENERGY_model.xlsx
+++ b/outputs/JSWENERGY_model.xlsx
@@ -82,7 +82,7 @@
     <t>India 10Y G-sec yield</t>
   </si>
   <si>
-    <t>Trading Economics, 25-Sep-2026</t>
+    <t>Investing.com historical close, 14-Aug-2026</t>
   </si>
   <si>
     <t>Sovereign default spread</t>
@@ -106,7 +106,7 @@
     <t>FY27 fraction remaining</t>
   </si>
   <si>
-    <t>Valuation date 25-Sep-2026</t>
+    <t>Valuation date 14-Aug-2026</t>
   </si>
   <si>
     <t>Weight on 12m DCF in target (non-regulated)</t>
@@ -145,7 +145,7 @@
     <t>Share price (Rs)</t>
   </si>
   <si>
-    <t>NSE close 2026-09-25</t>
+    <t>NSE close 2026-08-14</t>
   </si>
   <si>
     <t>Shares outstanding (crore)</t>
@@ -595,7 +595,7 @@
     <t>Blue = input, black = formula. Change Inputs or the guided-capex row on Model.</t>
   </si>
   <si>
-    <t>Prices as of 2026-09-25. Student research exercise, not investment advice.</t>
+    <t>Prices as of 2026-08-14. Student research exercise, not investment advice.</t>
   </si>
   <si>
     <t>Listed power comps, FY26A</t>
@@ -2107,7 +2107,7 @@
         <v>4</v>
       </c>
       <c r="C4" s="8">
-        <v>0.0711</v>
+        <v>0.06762</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>5</v>
@@ -2151,7 +2151,7 @@
         <v>12</v>
       </c>
       <c r="C8" s="9">
-        <v>0.51</v>
+        <v>0.6273972602739726</v>
       </c>
       <c r="D8" s="7" t="s">
         <v>13</v>
@@ -2184,7 +2184,7 @@
         <v>18</v>
       </c>
       <c r="C11" s="9">
-        <v>0.805</v>
+        <v>0.823</v>
       </c>
       <c r="D11" s="7" t="s">
         <v>19</v>
@@ -2226,7 +2226,7 @@
         <v>25</v>
       </c>
       <c r="C15" s="10">
-        <v>506.55</v>
+        <v>560</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>26</v>
@@ -2270,7 +2270,7 @@
         <v>32</v>
       </c>
       <c r="C19" s="11">
-        <v>14.14910340468798</v>
+        <v>14.5704823139073</v>
       </c>
       <c r="D19" s="7" t="s">
         <v>33</v>
@@ -6127,19 +6127,19 @@
         <v>188</v>
       </c>
       <c r="C4" s="5">
-        <v>390997.185143875</v>
+        <v>395818.358820125</v>
       </c>
       <c r="D4" s="5">
-        <v>444740.665143875</v>
+        <v>449561.838820125</v>
       </c>
       <c r="E4" s="11">
-        <v>22.45484525617868</v>
+        <v>22.69826511259845</v>
       </c>
       <c r="F4" s="11">
-        <v>30.14395074734986</v>
+        <v>30.5156394125453</v>
       </c>
       <c r="G4" s="11">
-        <v>6.021177220134515</v>
+        <v>6.095421082281673</v>
       </c>
       <c r="H4" s="6">
         <v>0.2138946604663434</v>
@@ -6159,19 +6159,19 @@
         <v>190</v>
       </c>
       <c r="C5" s="5">
-        <v>316693.11593644</v>
+        <v>326166.758749358</v>
       </c>
       <c r="D5" s="5">
-        <v>589225.82593644</v>
+        <v>598699.468749358</v>
       </c>
       <c r="E5" s="11">
-        <v>10.62855488900105</v>
+        <v>10.7994420568808</v>
       </c>
       <c r="F5" s="11">
-        <v>11.49688215844188</v>
+        <v>11.84080297500029</v>
       </c>
       <c r="G5" s="11">
-        <v>1.55871321384632</v>
+        <v>1.605340979000266</v>
       </c>
       <c r="H5" s="6">
         <v>0.1422657890183784</v>
@@ -6191,19 +6191,19 @@
         <v>192</v>
       </c>
       <c r="C6" s="5">
-        <v>250651.27292205</v>
+        <v>247442.564604495</v>
       </c>
       <c r="D6" s="5">
-        <v>393788.9629220501</v>
+        <v>390580.254604495</v>
       </c>
       <c r="E6" s="11">
-        <v>11.99442487045932</v>
+        <v>11.89669076800874</v>
       </c>
       <c r="F6" s="11">
-        <v>15.73651889264503</v>
+        <v>15.53506809420486</v>
       </c>
       <c r="G6" s="11">
-        <v>2.494191423587976</v>
+        <v>2.462262071412174</v>
       </c>
       <c r="H6" s="6">
         <v>0.1649228347924227</v>
@@ -6223,19 +6223,19 @@
         <v>194</v>
       </c>
       <c r="C7" s="5">
-        <v>213572.8602573</v>
+        <v>222039.345694</v>
       </c>
       <c r="D7" s="5">
-        <v>322958.8602573</v>
+        <v>331425.345694</v>
       </c>
       <c r="E7" s="11">
-        <v>29.94518871184979</v>
+        <v>30.73021285989801</v>
       </c>
       <c r="F7" s="11">
-        <v>107.4850831692501</v>
+        <v>111.7460219899346</v>
       </c>
       <c r="G7" s="11">
-        <v>10.69736339881292</v>
+        <v>11.12142978682695</v>
       </c>
       <c r="H7" s="6">
         <v>0.1237929100990592</v>
@@ -6255,19 +6255,19 @@
         <v>196</v>
       </c>
       <c r="C8" s="5">
-        <v>117428.72835225</v>
+        <v>122077.947393135</v>
       </c>
       <c r="D8" s="5">
-        <v>195874.79835225</v>
+        <v>200524.017393135</v>
       </c>
       <c r="E8" s="11">
-        <v>14.75961105811544</v>
+        <v>15.10994027527202</v>
       </c>
       <c r="F8" s="11">
-        <v>22.94426110829425</v>
+        <v>23.85266654809203</v>
       </c>
       <c r="G8" s="11">
-        <v>2.975289559953633</v>
+        <v>3.093086738449756</v>
       </c>
       <c r="H8" s="6">
         <v>0.1359200095606103</v>
@@ -6287,19 +6287,19 @@
         <v>198</v>
       </c>
       <c r="C9" s="5">
-        <v>92818.85147831999</v>
+        <v>102612.884864</v>
       </c>
       <c r="D9" s="5">
-        <v>164481.69147832</v>
+        <v>174275.724864</v>
       </c>
       <c r="E9" s="11">
-        <v>16.33707702406834</v>
+        <v>17.30986540166866</v>
       </c>
       <c r="F9" s="11">
-        <v>33.60566671916003</v>
+        <v>37.15165997972484</v>
       </c>
       <c r="G9" s="11">
-        <v>3.018401075682742</v>
+        <v>3.336895868882313</v>
       </c>
       <c r="H9" s="6">
         <v>0.0950578193832599</v>
@@ -6319,19 +6319,19 @@
         <v>200</v>
       </c>
       <c r="C10" s="5">
-        <v>76342.264518</v>
+        <v>77246.31765045</v>
       </c>
       <c r="D10" s="5">
-        <v>132109.384518</v>
+        <v>133013.43765045</v>
       </c>
       <c r="E10" s="11">
-        <v>32.24539529362949</v>
+        <v>32.46605751780572</v>
       </c>
       <c r="F10" s="11">
-        <v>18.09058400900474</v>
+        <v>18.30481460911138</v>
       </c>
       <c r="G10" s="11">
-        <v>1.842369489055675</v>
+        <v>1.864187022478703</v>
       </c>
       <c r="H10" s="6">
         <v>0.1040626348560508</v>
@@ -6351,19 +6351,19 @@
         <v>196</v>
       </c>
       <c r="C11" s="5">
-        <v>63219.73850477999</v>
+        <v>65966.01281412999</v>
       </c>
       <c r="D11" s="5">
-        <v>75504.74850477999</v>
+        <v>78251.02281412999</v>
       </c>
       <c r="E11" s="11">
-        <v>13.53859575126053</v>
+        <v>14.03102435254258</v>
       </c>
       <c r="F11" s="11">
-        <v>25.60540239156743</v>
+        <v>26.71770466347914</v>
       </c>
       <c r="G11" s="11">
-        <v>3.314272005493053</v>
+        <v>3.458244446350196</v>
       </c>
       <c r="H11" s="6">
         <v>0.1345870809484873</v>
@@ -6383,19 +6383,19 @@
         <v>203</v>
       </c>
       <c r="C12" s="5">
-        <v>36406.144169295</v>
+        <v>38151.919660026</v>
       </c>
       <c r="D12" s="5">
-        <v>67334.034169295</v>
+        <v>69079.80966002599</v>
       </c>
       <c r="E12" s="11">
-        <v>12.11479564039133</v>
+        <v>12.42889702411407</v>
       </c>
       <c r="F12" s="11">
-        <v>9.659364332527195</v>
+        <v>10.12255761741205</v>
       </c>
       <c r="G12" s="11">
-        <v>1.691342353974216</v>
+        <v>1.772446906389129</v>
       </c>
       <c r="H12" s="6">
         <v>0.1872888093818326</v>
@@ -6415,19 +6415,19 @@
         <v>200</v>
       </c>
       <c r="C13" s="5">
-        <v>24270.4150008</v>
+        <v>26270.680744875</v>
       </c>
       <c r="D13" s="5">
-        <v>54422.8450008</v>
+        <v>56423.11074487499</v>
       </c>
       <c r="E13" s="11">
-        <v>16.19245611448974</v>
+        <v>16.78759617520827</v>
       </c>
       <c r="F13" s="11">
-        <v>37.8043847364486</v>
+        <v>40.92006346553738</v>
       </c>
       <c r="G13" s="11">
-        <v>1.704502774127397</v>
+        <v>1.844980739158298</v>
       </c>
       <c r="H13" s="6">
         <v>0.045182630727004</v>
@@ -6447,19 +6447,19 @@
         <v>196</v>
       </c>
       <c r="C14" s="5">
-        <v>18539.42803398</v>
+        <v>21453.03183912</v>
       </c>
       <c r="D14" s="5">
-        <v>35265.42803398</v>
+        <v>38179.03183912001</v>
       </c>
       <c r="E14" s="11">
-        <v>9.731078375822296</v>
+        <v>10.53505293573952</v>
       </c>
       <c r="F14" s="11">
-        <v>11.45823735103832</v>
+        <v>13.25898135915946</v>
       </c>
       <c r="G14" s="11">
-        <v>1.47960319505028</v>
+        <v>1.712133426905028</v>
       </c>
       <c r="H14" s="6">
         <v>0.1318663406682966</v>
@@ -6479,19 +6479,19 @@
         <v>188</v>
       </c>
       <c r="C15" s="5">
-        <v>10876.439158449</v>
+        <v>11918.164900153</v>
       </c>
       <c r="D15" s="5">
-        <v>13512.489158449</v>
+        <v>14554.214900153</v>
       </c>
       <c r="E15" s="11">
-        <v>9.884776268068032</v>
+        <v>10.64682874919751</v>
       </c>
       <c r="F15" s="11">
-        <v>24.11627307860089</v>
+        <v>26.42608625311087</v>
       </c>
       <c r="G15" s="11">
-        <v>0.8542600658536758</v>
+        <v>0.9360795554628496</v>
       </c>
       <c r="H15" s="6">
         <v>0.0360612481509615</v>
@@ -6511,16 +6511,16 @@
         <v>188</v>
       </c>
       <c r="C16" s="5">
-        <v>8507.280877061999</v>
+        <v>9504.001679868001</v>
       </c>
       <c r="D16" s="5">
-        <v>22815.030877062</v>
+        <v>23811.751679868</v>
       </c>
       <c r="E16" s="11">
-        <v>9.646947516728121</v>
+        <v>10.0683939449759</v>
       </c>
       <c r="G16" s="11">
-        <v>0.5303791070487531</v>
+        <v>0.5925188079718205</v>
       </c>
       <c r="H16" s="6">
         <v>-0.0208172468110078</v>
@@ -6540,19 +6540,19 @@
         <v>209</v>
       </c>
       <c r="C17" s="5">
-        <v>4590.793050389</v>
+        <v>4779.646359187001</v>
       </c>
       <c r="D17" s="5">
-        <v>2852.353050389</v>
+        <v>3041.206359187</v>
       </c>
       <c r="E17" s="11">
-        <v>3.197705213440583</v>
+        <v>3.409424169492153</v>
       </c>
       <c r="F17" s="11">
-        <v>6.402779707655509</v>
+        <v>6.666173443775454</v>
       </c>
       <c r="G17" s="11">
-        <v>0.7675627905682997</v>
+        <v>0.7991383312467816</v>
       </c>
       <c r="H17" s="6">
         <v>0.1216697777023587</v>

</xml_diff>